<commit_message>
feat: update chart containers to use card styling for improved UI consistency; add CSS for Chart 6 area chart
</commit_message>
<xml_diff>
--- a/project1/Typo.xlsx
+++ b/project1/Typo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fanshawe college\3171_UI&amp;DataVisualization\week5\Info_3171_group_project\project1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE39B51-A86E-4AD2-B5C4-DD273C888B62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4DD2D52-749C-4FDB-B91D-F18E4202B20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12588" yWindow="0" windowWidth="10530" windowHeight="13758" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
+    <workbookView xWindow="11526" yWindow="30" windowWidth="11712" windowHeight="8790" xr2:uid="{C05D5FBD-05C5-4BAC-BB6B-32F74FCC0EAE}"/>
   </bookViews>
   <sheets>
     <sheet name="Typo" sheetId="1" r:id="rId1"/>

</xml_diff>